<commit_message>
Update spreadsheet with final benchmark numbers
</commit_message>
<xml_diff>
--- a/benchmarks/TurboQuant-MLX-Results.xlsx
+++ b/benchmarks/TurboQuant-MLX-Results.xlsx
@@ -73,7 +73,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -99,6 +99,9 @@
     <xf numFmtId="168" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -464,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1220,6 +1223,118 @@
         <v>52</v>
       </c>
       <c r="N13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Qwen2.5-32B</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Dense base</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>32</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>FINAL: Dual+T1+T4</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>1.4141</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.4154</v>
+      </c>
+      <c r="G14" s="9">
+        <f>IF(F14="","",ABS(F14-E14))</f>
+        <v/>
+      </c>
+      <c r="H14" s="10">
+        <f>IF(F14="","",ABS(F14-E14)/E14*100)</f>
+        <v/>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>&lt;0.1%</t>
+        </is>
+      </c>
+      <c r="J14">
+        <f>IF(F14="","PENDING",IF(H14&lt;VALUE(SUBSTITUTE(SUBSTITUTE(I14,"&lt;",""),"%","")),"PASS","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="K14" s="11">
+        <f>IF(L14="","",L14/M14)</f>
+        <v/>
+      </c>
+      <c r="L14" t="n">
+        <v>34</v>
+      </c>
+      <c r="M14" t="n">
+        <v>61</v>
+      </c>
+      <c r="N14" t="n">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Qwen3.5-27B</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>27</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>FINAL: Dual+T1+T4</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>1.4531</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1.4557</v>
+      </c>
+      <c r="G15" s="9">
+        <f>IF(F15="","",ABS(F15-E15))</f>
+        <v/>
+      </c>
+      <c r="H15" s="10">
+        <f>IF(F15="","",ABS(F15-E15)/E15*100)</f>
+        <v/>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>&lt;0.2%</t>
+        </is>
+      </c>
+      <c r="J15">
+        <f>IF(F15="","PENDING",IF(H15&lt;VALUE(SUBSTITUTE(SUBSTITUTE(I15,"&lt;",""),"%","")),"PASS","FAIL"))</f>
+        <v/>
+      </c>
+      <c r="K15" s="11">
+        <f>IF(L15="","",L15/M15)</f>
+        <v/>
+      </c>
+      <c r="L15" t="n">
+        <v>29</v>
+      </c>
+      <c r="M15" t="n">
+        <v>52</v>
+      </c>
+      <c r="N15" t="n">
+        <v>197</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1534,7 +1649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1590,7 +1705,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>0.28</v>
+        <v>0.302</v>
       </c>
       <c r="C2" s="7">
         <f>IF(B2="","",1000/B2)</f>
@@ -1620,7 +1735,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.21</v>
+        <v>0.219</v>
       </c>
       <c r="C3" s="7">
         <f>IF(B3="","",1000/B3)</f>
@@ -1646,7 +1761,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TQ8 pre-optimization</t>
+          <t>TQ8 pre-optimization (Phase 1)</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
@@ -1766,11 +1881,11 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TQ8 final (best run)</t>
+          <t>TQ8 FINAL (dual rot default)</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>1.81</v>
+        <v>1.49</v>
       </c>
       <c r="C8" s="7">
         <f>IF(B8="","",1000/B8)</f>
@@ -1826,11 +1941,11 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TQ8 E2E post-opt (real layer)</t>
+          <t>TQ8 E2E FINAL (real layer)</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>21.6</v>
+        <v>21.1</v>
       </c>
       <c r="C10" s="7">
         <f>IF(B10="","",1000/B10)</f>
@@ -1851,6 +1966,40 @@
       </c>
       <c r="G10" s="2" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Dequant throughput pre-opt</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>4096x4096</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1.33 GB/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Dequant throughput FINAL</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>4096x4096</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>17.35 GB/s</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>